<commit_message>
data: publish 2026-09-23 sampler-linked operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-23-182路.xlsx
+++ b/data/export/2026-09-23-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC9"/>
+  <dimension ref="A1:AC17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -637,24 +637,24 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>07:10</t>
+          <t>07:16</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>65分钟</t>
+          <t>71分钟</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
       <c r="K2" s="2" t="inlineStr"/>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站德川路华夏东路 ETA 1分钟；叠加该车自身同类时段从该站到终点历史中位数47分钟，约±5分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -693,12 +693,12 @@
       </c>
       <c r="W2" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X2" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y2" s="2" t="inlineStr">
@@ -708,22 +708,22 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
         <is>
-          <t>65.0</t>
+          <t>79.5</t>
         </is>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>1/8</t>
+          <t>3/13</t>
         </is>
       </c>
     </row>
@@ -756,24 +756,24 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>70分钟</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
       <c r="K3" s="2" t="inlineStr"/>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>06:21采样：该车到重点站博兴路东陆路 ETA 3分钟；叠加该车自身同类时段从该站到终点历史中位数56分钟，约±5分钟</t>
+          <t>SHMAAS终点ETA近站估算，约±5分钟</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -812,12 +812,12 @@
       </c>
       <c r="W3" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X3" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y3" s="2" t="inlineStr">
@@ -837,12 +837,12 @@
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>70.0</t>
+          <t>72.0</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>2/8</t>
+          <t>2/13</t>
         </is>
       </c>
     </row>
@@ -875,29 +875,29 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>07:31</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>72分钟</t>
+          <t>77分钟</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>06:11</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="W4" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X4" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y4" s="2" t="inlineStr">
@@ -946,22 +946,22 @@
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA4" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB4" s="2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>82.5</t>
         </is>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>6/13</t>
         </is>
       </c>
     </row>
@@ -994,29 +994,29 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>07:54</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>80分钟</t>
+          <t>83分钟</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
       <c r="K5" s="2" t="inlineStr"/>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数80分钟估算，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±4分钟</t>
         </is>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="W5" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X5" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y5" s="2" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>80.0</t>
+          <t>83.0</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>5/8</t>
+          <t>7/13</t>
         </is>
       </c>
     </row>
@@ -1118,26 +1118,22 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>88分钟</t>
+          <t>81分钟</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
       <c r="K6" s="2" t="inlineStr"/>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数88分钟估算，约±8分钟</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
+          <t>SHMAAS末次终点ETA推算：07:20采样，终点ETA 35分钟</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -1145,7 +1141,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1169,12 +1165,12 @@
       </c>
       <c r="W6" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="X6" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>末次终点ETA兜底</t>
         </is>
       </c>
       <c r="Y6" s="2" t="inlineStr">
@@ -1184,22 +1180,22 @@
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AA6" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="AB6" s="2" t="inlineStr">
         <is>
-          <t>88.0</t>
+          <t>81.5</t>
         </is>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
-          <t>6/8</t>
+          <t>4/13</t>
         </is>
       </c>
     </row>
@@ -1237,24 +1233,24 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:58</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>72分钟</t>
+          <t>71分钟</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
       <c r="K7" s="2" t="inlineStr"/>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±8分钟</t>
+          <t>07:20采样：该车到重点站唐陆公路锦绣东路 ETA 10分钟；叠加该车自身同类时段从该站到终点历史中位数28分钟，约±9分钟</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>9</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -1264,7 +1260,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1293,7 +1289,7 @@
       </c>
       <c r="X7" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y7" s="2" t="inlineStr">
@@ -1313,12 +1309,12 @@
       </c>
       <c r="AB7" s="2" t="inlineStr">
         <is>
-          <t>72.0</t>
+          <t>71.0</t>
         </is>
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>3/8</t>
+          <t>1/13</t>
         </is>
       </c>
     </row>
@@ -1356,22 +1352,26 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>08:24</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>待确认</t>
+          <t>89分钟</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr"/>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>尚无满足±5分钟标准的终点ETA</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr"/>
+          <t>07:20采样：该车到重点站东陆路金海路 ETA 6分钟；叠加该车自身同类时段从该站到终点历史中位数58分钟，约±15分钟</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="inlineStr">
         <is>
           <t>06:01</t>
@@ -1379,7 +1379,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1403,17 +1403,17 @@
       </c>
       <c r="W8" s="2" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="X8" s="2" t="inlineStr">
         <is>
-          <t>证据不足</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y8" s="2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
       <c r="Z8" s="2" t="inlineStr">
@@ -1423,13 +1423,17 @@
       </c>
       <c r="AA8" s="2" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AB8" s="2" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB8" s="2" t="inlineStr">
+        <is>
+          <t>89.0</t>
+        </is>
+      </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>—/8</t>
+          <t>10/13</t>
         </is>
       </c>
     </row>
@@ -1437,24 +1441,24 @@
       <c r="A9" s="2" t="inlineStr"/>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>沪A32298D</t>
+          <t>沪A12050A</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>金杨路金口路</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>07:15</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>川沙客运站</t>
-        </is>
-      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>全程车</t>
@@ -1467,34 +1471,34 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>08:44</t>
+          <t>08:26</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>89分钟</t>
+          <t>87分钟</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr"/>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数89分钟估算，约±10分钟</t>
+          <t>07:20采样：该车到重点站新德西路德翔路 ETA 1分钟；叠加该车自身同类时段从该站到终点历史中位数65分钟，约±13分钟</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>13</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>06:01</t>
+          <t>06:32</t>
         </is>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>06:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1508,47 +1512,999 @@
       <c r="T9" s="2" t="inlineStr"/>
       <c r="U9" s="2" t="inlineStr">
         <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA9" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB9" s="2" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="AC9" s="2" t="inlineStr">
+        <is>
+          <t>8/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>沪A35717D</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>89分钟</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>07:20采样：该车到重点站新川路妙境路 ETA 6分钟；叠加该车自身同类时段从该站到终点历史中位数74分钟，约±7分钟</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>07:12</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y10" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA10" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB10" s="2" t="inlineStr">
+        <is>
+          <t>89.0</t>
+        </is>
+      </c>
+      <c r="AC10" s="2" t="inlineStr">
+        <is>
+          <t>10/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>沪A32298D</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
           <t>07:15</t>
         </is>
       </c>
-      <c r="V9" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>93分钟</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>07:20采样：该车到重点站长岛路台儿庄路 ETA 11分钟；叠加该车自身同类时段从该站到终点历史中位数77分钟，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
         <is>
           <t>计划发车</t>
         </is>
       </c>
-      <c r="W9" s="2" t="inlineStr">
+      <c r="W11" s="2" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="X9" s="2" t="inlineStr">
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>同车重点站剩余时间</t>
+        </is>
+      </c>
+      <c r="Y11" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA11" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB11" s="2" t="inlineStr">
+        <is>
+          <t>93.0</t>
+        </is>
+      </c>
+      <c r="AC11" s="2" t="inlineStr">
+        <is>
+          <t>13/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr"/>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>沪A31073D</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>08:51</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>87分钟</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数87分钟估算，约±6分钟</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr"/>
+      <c r="R12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>07:24</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
         <is>
           <t>同车历史全程时间</t>
         </is>
       </c>
-      <c r="Y9" s="2" t="inlineStr">
+      <c r="Y12" s="2" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="Z9" s="2" t="inlineStr">
+      <c r="Z12" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AA9" s="2" t="inlineStr">
+      <c r="AA12" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="AB9" s="2" t="inlineStr">
-        <is>
-          <t>89.0</t>
-        </is>
-      </c>
-      <c r="AC9" s="2" t="inlineStr">
-        <is>
-          <t>7/8</t>
+      <c r="AB12" s="2" t="inlineStr">
+        <is>
+          <t>87.0</t>
+        </is>
+      </c>
+      <c r="AC12" s="2" t="inlineStr">
+        <is>
+          <t>8/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>09:03</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>88分钟</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数88分钟估算，约±10分钟</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="inlineStr"/>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y13" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB13" s="2" t="inlineStr">
+        <is>
+          <t>79.5</t>
+        </is>
+      </c>
+      <c r="AC13" s="2" t="inlineStr">
+        <is>
+          <t>3/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>沪A55712D</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>09:07</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>91分钟</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数91分钟估算，约±15分钟</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>07:02</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr"/>
+      <c r="R14" s="2" t="inlineStr"/>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y14" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA14" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB14" s="2" t="inlineStr">
+        <is>
+          <t>91.0</t>
+        </is>
+      </c>
+      <c r="AC14" s="2" t="inlineStr">
+        <is>
+          <t>12/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>沪A02126A</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>82分钟</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数82分钟估算，约±13分钟</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr"/>
+      <c r="R15" s="2" t="inlineStr"/>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>07:48</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y15" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AA15" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AB15" s="2" t="inlineStr">
+        <is>
+          <t>82.0</t>
+        </is>
+      </c>
+      <c r="AC15" s="2" t="inlineStr">
+        <is>
+          <t>5/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>沪A68870D</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>09:23</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>88分钟</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数88分钟估算，约±6分钟</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr"/>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y16" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB16" s="2" t="inlineStr">
+        <is>
+          <t>82.5</t>
+        </is>
+      </c>
+      <c r="AC16" s="2" t="inlineStr">
+        <is>
+          <t>6/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>沪A67026D</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>09:37</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>82分钟</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数82分钟估算，约±9分钟</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr"/>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y17" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AA17" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="AB17" s="2" t="inlineStr">
+        <is>
+          <t>81.5</t>
+        </is>
+      </c>
+      <c r="AC17" s="2" t="inlineStr">
+        <is>
+          <t>4/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: publish 2026-09-23 rolling operations analysis
</commit_message>
<xml_diff>
--- a/data/export/2026-09-23-182路.xlsx
+++ b/data/export/2026-09-23-182路.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC55"/>
+  <dimension ref="A1:AC58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -669,7 +669,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA2" s="2" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -788,7 +788,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA3" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB3" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -1026,7 +1026,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -1065,22 +1065,22 @@
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB5" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>74.8</t>
         </is>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="AC7" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="AC8" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -1621,7 +1621,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1670,7 +1670,7 @@
       </c>
       <c r="AB10" s="2" t="inlineStr">
         <is>
-          <t>79.2</t>
+          <t>78.5</t>
         </is>
       </c>
       <c r="AC10" s="2" t="inlineStr">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1908,12 +1908,12 @@
       </c>
       <c r="AB12" s="2" t="inlineStr">
         <is>
-          <t>78.5</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC12" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -2017,7 +2017,7 @@
       </c>
       <c r="Z13" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA13" s="2" t="inlineStr">
@@ -2032,7 +2032,7 @@
       </c>
       <c r="AC13" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -2146,12 +2146,12 @@
       </c>
       <c r="AB14" s="2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC14" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -2216,7 +2216,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -2265,12 +2265,12 @@
       </c>
       <c r="AB15" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC15" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -2389,7 +2389,7 @@
       </c>
       <c r="AC16" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -2493,22 +2493,22 @@
       </c>
       <c r="Z17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA17" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2573,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2612,22 +2612,22 @@
       </c>
       <c r="Z18" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA18" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB18" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>74.8</t>
         </is>
       </c>
       <c r="AC18" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -2811,7 +2811,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="AC20" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="AC21" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -3099,7 +3099,7 @@
       </c>
       <c r="AC22" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3451,7 +3451,7 @@
       </c>
       <c r="AB25" s="2" t="inlineStr">
         <is>
-          <t>79.2</t>
+          <t>78.5</t>
         </is>
       </c>
       <c r="AC25" s="2" t="inlineStr">
@@ -3521,7 +3521,7 @@
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -3570,12 +3570,12 @@
       </c>
       <c r="AB26" s="2" t="inlineStr">
         <is>
-          <t>78.5</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC26" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA27" s="2" t="inlineStr">
@@ -3694,7 +3694,7 @@
       </c>
       <c r="AC27" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3808,12 +3808,12 @@
       </c>
       <c r="AB28" s="2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC28" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3927,12 +3927,12 @@
       </c>
       <c r="AB29" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC29" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="AC30" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -4116,7 +4116,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -4155,22 +4155,22 @@
       </c>
       <c r="Z31" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA31" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB31" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="AC31" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -4354,7 +4354,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -4393,22 +4393,22 @@
       </c>
       <c r="Z33" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA33" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB33" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>74.8</t>
         </is>
       </c>
       <c r="AC33" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -4473,7 +4473,7 @@
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P34" s="2" t="inlineStr">
@@ -4527,7 +4527,7 @@
       </c>
       <c r="AC34" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="AC35" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P36" s="2" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="AC36" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
@@ -4949,7 +4949,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4998,7 +4998,7 @@
       </c>
       <c r="AB38" s="2" t="inlineStr">
         <is>
-          <t>79.2</t>
+          <t>78.5</t>
         </is>
       </c>
       <c r="AC38" s="2" t="inlineStr">
@@ -5068,7 +5068,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -5107,7 +5107,7 @@
       </c>
       <c r="Z39" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA39" s="2" t="inlineStr">
@@ -5122,7 +5122,7 @@
       </c>
       <c r="AC39" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>8/14</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -5236,12 +5236,12 @@
       </c>
       <c r="AB40" s="2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC40" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
       </c>
       <c r="AC41" s="2" t="inlineStr">
         <is>
-          <t>9/14</t>
+          <t>10/14</t>
         </is>
       </c>
     </row>
@@ -5425,7 +5425,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P42" s="2" t="inlineStr">
@@ -5474,12 +5474,12 @@
       </c>
       <c r="AB42" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC42" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5717,7 +5717,7 @@
       </c>
       <c r="AC44" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -5836,7 +5836,7 @@
       </c>
       <c r="AC45" s="2" t="inlineStr">
         <is>
-          <t>1/14</t>
+          <t>2/14</t>
         </is>
       </c>
     </row>
@@ -5869,27 +5869,31 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:53</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>76分钟</t>
+          <t>73分钟</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS末次终点ETA推算：13:21采样，终点ETA 34分钟</t>
-        </is>
-      </c>
-      <c r="M46" s="2" t="inlineStr"/>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
           <t>06:41</t>
@@ -5897,7 +5901,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P46" s="2" t="inlineStr">
@@ -5921,12 +5925,12 @@
       </c>
       <c r="W46" s="2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X46" s="2" t="inlineStr">
         <is>
-          <t>末次终点ETA兜底</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y46" s="2" t="inlineStr">
@@ -5946,7 +5950,7 @@
       </c>
       <c r="AB46" s="2" t="inlineStr">
         <is>
-          <t>79.2</t>
+          <t>78.5</t>
         </is>
       </c>
       <c r="AC46" s="2" t="inlineStr">
@@ -5989,24 +5993,24 @@
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:53</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
         <is>
-          <t>70分钟</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr"/>
       <c r="L47" s="2" t="inlineStr">
         <is>
-          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
+          <t>SHMAAS终点近站ETA直接确认，约±2分钟</t>
         </is>
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N47" s="2" t="inlineStr">
@@ -6016,7 +6020,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P47" s="2" t="inlineStr">
@@ -6065,12 +6069,12 @@
       </c>
       <c r="AB47" s="2" t="inlineStr">
         <is>
-          <t>78.5</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC47" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -6103,29 +6107,29 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
         <is>
-          <t>14:13</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="I48" s="2" t="inlineStr">
         <is>
-          <t>73分钟</t>
+          <t>72分钟</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>13:21采样：该车到重点站东陆路金海路 ETA 4分钟；叠加该车自身同类时段从该站到终点历史中位数48分钟，约±9分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±5分钟</t>
         </is>
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N48" s="2" t="inlineStr">
@@ -6135,7 +6139,7 @@
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P48" s="2" t="inlineStr">
@@ -6159,12 +6163,12 @@
       </c>
       <c r="W48" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X48" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y48" s="2" t="inlineStr">
@@ -6184,12 +6188,12 @@
       </c>
       <c r="AB48" s="2" t="inlineStr">
         <is>
-          <t>77.0</t>
+          <t>76.8</t>
         </is>
       </c>
       <c r="AC48" s="2" t="inlineStr">
         <is>
-          <t>7/14</t>
+          <t>6/14</t>
         </is>
       </c>
     </row>
@@ -6222,7 +6226,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+          <t>已取得可靠同向线路终点ETA，按全程车保护</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -6239,12 +6243,12 @@
       <c r="K49" s="2" t="inlineStr"/>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>13:21采样：该车到重点站新川路妙境路 ETA 0分钟；叠加该车自身同类时段从该站到终点历史中位数63分钟，约±5分钟</t>
+          <t>SHMAAS多次终点ETA一致估算，约±3分钟</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="N49" s="2" t="inlineStr">
@@ -6254,7 +6258,7 @@
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P49" s="2" t="inlineStr">
@@ -6278,12 +6282,12 @@
       </c>
       <c r="W49" s="2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="X49" s="2" t="inlineStr">
         <is>
-          <t>同车重点站剩余时间</t>
+          <t>终点ETA确认/一致估算</t>
         </is>
       </c>
       <c r="Y49" s="2" t="inlineStr">
@@ -6293,22 +6297,22 @@
       </c>
       <c r="Z49" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA49" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB49" s="2" t="inlineStr">
         <is>
-          <t>78.8</t>
+          <t>77.4</t>
         </is>
       </c>
       <c r="AC49" s="2" t="inlineStr">
         <is>
-          <t>11/14</t>
+          <t>9/14</t>
         </is>
       </c>
     </row>
@@ -6346,24 +6350,24 @@
       </c>
       <c r="H50" s="2" t="inlineStr">
         <is>
-          <t>14:34</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="I50" s="2" t="inlineStr">
         <is>
-          <t>69分钟</t>
+          <t>60分钟</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr"/>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数69分钟估算，约±8分钟</t>
+          <t>13:52采样：该车到重点站唐陆公路锦绣东路 ETA 4分钟；叠加该车自身同类时段从该站到终点历史中位数29分钟，约±5分钟</t>
         </is>
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -6373,7 +6377,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P50" s="2" t="inlineStr">
@@ -6402,7 +6406,7 @@
       </c>
       <c r="X50" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车重点站剩余时间</t>
         </is>
       </c>
       <c r="Y50" s="2" t="inlineStr">
@@ -6422,12 +6426,12 @@
       </c>
       <c r="AB50" s="2" t="inlineStr">
         <is>
-          <t>74.8</t>
+          <t>72.5</t>
         </is>
       </c>
       <c r="AC50" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>1/14</t>
         </is>
       </c>
     </row>
@@ -6465,24 +6469,24 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:43</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>73分钟</t>
+          <t>68分钟</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr">
         <is>
-          <t>按该车自身同方向、同类时段历史全程时间中位数73分钟估算，约±6分钟</t>
+          <t>同车下一次反向发车15:00，减去该车自身同类时段历史终点停站中位数17分钟，约±10分钟</t>
         </is>
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>10</t>
         </is>
       </c>
       <c r="N51" s="2" t="inlineStr">
@@ -6492,7 +6496,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -6521,7 +6525,7 @@
       </c>
       <c r="X51" s="2" t="inlineStr">
         <is>
-          <t>同车历史全程时间</t>
+          <t>同车反向发车反推</t>
         </is>
       </c>
       <c r="Y51" s="2" t="inlineStr">
@@ -6531,22 +6535,22 @@
       </c>
       <c r="Z51" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AA51" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="AB51" s="2" t="inlineStr">
         <is>
-          <t>76.2</t>
+          <t>74.8</t>
         </is>
       </c>
       <c r="AC51" s="2" t="inlineStr">
         <is>
-          <t>5/14</t>
+          <t>4/14</t>
         </is>
       </c>
     </row>
@@ -6611,7 +6615,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -6665,7 +6669,7 @@
       </c>
       <c r="AC52" s="2" t="inlineStr">
         <is>
-          <t>2/14</t>
+          <t>3/14</t>
         </is>
       </c>
     </row>
@@ -6730,7 +6734,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -6784,7 +6788,7 @@
       </c>
       <c r="AC53" s="2" t="inlineStr">
         <is>
-          <t>4/14</t>
+          <t>5/14</t>
         </is>
       </c>
     </row>
@@ -6849,7 +6853,7 @@
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P54" s="2" t="inlineStr">
@@ -6898,12 +6902,12 @@
       </c>
       <c r="AB54" s="2" t="inlineStr">
         <is>
-          <t>78.5</t>
+          <t>78.0</t>
         </is>
       </c>
       <c r="AC54" s="2" t="inlineStr">
         <is>
-          <t>10/14</t>
+          <t>11/14</t>
         </is>
       </c>
     </row>
@@ -6968,7 +6972,7 @@
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:52</t>
         </is>
       </c>
       <c r="P55" s="2" t="inlineStr">
@@ -7026,6 +7030,359 @@
         </is>
       </c>
     </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr"/>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>沪A67983D</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>72分钟</t>
+        </is>
+      </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数72分钟估算，约±5分钟</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="P56" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q56" s="2" t="inlineStr"/>
+      <c r="R56" s="2" t="inlineStr"/>
+      <c r="S56" s="2" t="inlineStr"/>
+      <c r="T56" s="2" t="inlineStr"/>
+      <c r="U56" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="V56" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W56" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X56" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y56" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z56" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA56" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AB56" s="2" t="inlineStr">
+        <is>
+          <t>77.4</t>
+        </is>
+      </c>
+      <c r="AC56" s="2" t="inlineStr">
+        <is>
+          <t>9/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr"/>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>沪A68397D</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>待确认</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>尚无满足±5分钟标准的终点ETA</t>
+        </is>
+      </c>
+      <c r="M57" s="2" t="inlineStr"/>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="P57" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q57" s="2" t="inlineStr"/>
+      <c r="R57" s="2" t="inlineStr"/>
+      <c r="S57" s="2" t="inlineStr"/>
+      <c r="T57" s="2" t="inlineStr"/>
+      <c r="U57" s="2" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="V57" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W57" s="2" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="X57" s="2" t="inlineStr">
+        <is>
+          <t>证据不足</t>
+        </is>
+      </c>
+      <c r="Y57" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="Z57" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA57" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="AB57" s="2" t="inlineStr">
+        <is>
+          <t>77.0</t>
+        </is>
+      </c>
+      <c r="AC57" s="2" t="inlineStr">
+        <is>
+          <t>8/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr"/>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>沪A13735A</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>金杨路金口路</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>川沙客运站</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>全程车</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>未形成反向≥2站物理推进证据或可靠时空矛盾</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>16:14</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>74分钟</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr"/>
+      <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>按该车自身同方向、同类时段历史全程时间中位数74分钟估算，约±8分钟</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="P58" s="2" t="inlineStr">
+        <is>
+          <t>SHMAAS</t>
+        </is>
+      </c>
+      <c r="Q58" s="2" t="inlineStr"/>
+      <c r="R58" s="2" t="inlineStr"/>
+      <c r="S58" s="2" t="inlineStr"/>
+      <c r="T58" s="2" t="inlineStr"/>
+      <c r="U58" s="2" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="V58" s="2" t="inlineStr">
+        <is>
+          <t>计划发车</t>
+        </is>
+      </c>
+      <c r="W58" s="2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="X58" s="2" t="inlineStr">
+        <is>
+          <t>同车历史全程时间</t>
+        </is>
+      </c>
+      <c r="Y58" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="Z58" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AA58" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="AB58" s="2" t="inlineStr">
+        <is>
+          <t>74.8</t>
+        </is>
+      </c>
+      <c r="AC58" s="2" t="inlineStr">
+        <is>
+          <t>4/14</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>